<commit_message>
dashboard de precios terminada
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\big_data\matematicas\analisis_estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BF9B2D-D51D-4180-951F-7B977F1B93EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E97D849-8A5E-4878-84CD-3E3E9289203C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,12 @@
     <sheet name="3_Satisfaccion" sheetId="4" r:id="rId4"/>
     <sheet name="4_Probabilidad" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="154">
   <si>
     <t>ID_Venta</t>
   </si>
@@ -487,13 +493,25 @@
   </si>
   <si>
     <t>Dashboard 4: Probabilidad y Frecuencias (Canales)</t>
+  </si>
+  <si>
+    <t>18 Euros es el producto que más se ha comprado</t>
+  </si>
+  <si>
+    <t>Media y mediana no son parecida, esto inplica muchos valores extremos</t>
+  </si>
+  <si>
+    <t>Sobre todo en la parte alta, que distorciona la media.</t>
+  </si>
+  <si>
+    <t>El precio medio de nuestra tienda es 35 (Mediana)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -537,6 +555,13 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -601,7 +626,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -613,6 +638,7 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,6 +654,701 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.2</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.3</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Histograma de precios</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Histograma de precios</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{967C21E4-8A90-4B51-AE1E-E3C6500796EF}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5442</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>2720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>277585</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>179614</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Gráfico 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0AA995FD-664B-E2F9-51B8-25363624A18D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4250871" y="2266949"/>
+              <a:ext cx="4572000" cy="2767694"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-ES" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -922,6 +1643,7 @@
   <cols>
     <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.77734375" bestFit="1" customWidth="1"/>
@@ -2865,7 +3587,10 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>60.011904761904759</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -2877,7 +3602,10 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -2889,7 +3617,10 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2901,7 +3632,10 @@
       <c r="D8" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E8" s="4"/>
+      <c r="E8" s="4">
+        <f>_xlfn.STDEV.S(B5:B46)</f>
+        <v>63.23692269082472</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -2970,7 +3704,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -2978,7 +3712,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -2986,7 +3720,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -2994,7 +3728,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -3002,7 +3736,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -3010,7 +3744,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -3018,7 +3752,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -3026,7 +3760,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -3034,7 +3768,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -3042,7 +3776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3050,7 +3784,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3058,7 +3792,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -3066,36 +3800,48 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
       <c r="B29">
         <v>120</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D29" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>81</v>
       </c>
       <c r="B30">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D30" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>82</v>
       </c>
       <c r="B31">
         <v>12</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D31" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>83</v>
       </c>
       <c r="B32">
         <v>30</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
@@ -3212,6 +3958,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
panel de beneficios completado
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\big_data\matematicas\analisis_estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E97D849-8A5E-4878-84CD-3E3E9289203C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A673359-62BA-4936-8FDD-53D43C813C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -22,8 +22,6 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -656,15 +654,577 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Dispersión:</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-ES" baseline="0"/>
+              <a:t> Coste vs Beneficio</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'2_Beneficios'!$B$5:$B$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="42"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>80</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'2_Beneficios'!$C$5:$C$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="42"/>
+                <c:pt idx="0">
+                  <c:v>15.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-58C0-4957-935D-9E63E1CF4A18}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="642384847"/>
+        <c:axId val="642390607"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="642384847"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="642390607"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="642390607"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="642384847"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v1.2</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -721,6 +1281,46 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1268,6 +1868,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1317,8 +2433,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="4250871" y="2266949"/>
-              <a:ext cx="4572000" cy="2767694"/>
+              <a:off x="4257402" y="2243000"/>
+              <a:ext cx="4569823" cy="2737214"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -1346,6 +2462,47 @@
         </xdr:sp>
       </mc:Fallback>
     </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6482882-14F9-D2B6-0402-7B279345D293}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -4008,7 +5165,10 @@
       <c r="E5" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="4">
+        <f>AVERAGE(C5:C46)</f>
+        <v>32.511904761904759</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -4023,7 +5183,10 @@
       <c r="E6" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="4"/>
+      <c r="F6" s="4">
+        <f>_xlfn.STDEV.S(C5:C46)</f>
+        <v>20.550499399082351</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -4038,7 +5201,10 @@
       <c r="E7" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="4">
+        <f>MIN(C5:C46)</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -4053,7 +5219,10 @@
       <c r="E8" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="4">
+        <f>MAX(C5:C46)</f>
+        <v>120</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -4478,6 +5647,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Valoración de satisfacción terminada
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\big_data\matematicas\analisis_estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A673359-62BA-4936-8FDD-53D43C813C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C943EF-923D-4C91-B8C5-63BCC539387A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -1216,6 +1216,315 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES" baseline="0"/>
+              <a:t>Distribucción de Satisfacción</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$D$12:$D$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$E$12:$E$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3906-4089-BB78-7CE3909CC87A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1722854128"/>
+        <c:axId val="1722852208"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1722854128"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1722852208"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1722852208"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1722854128"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1360,6 +1669,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -2365,6 +2714,509 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -2488,6 +3340,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6482882-14F9-D2B6-0402-7B279345D293}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>6350</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A536012-38AD-6E43-3603-6841D2FA2270}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5658,7 +6551,7 @@
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
     <col min="2" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="4" max="4" width="60.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5691,7 +6584,10 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>4.2857142857142856</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -5703,7 +6599,10 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -5715,7 +6614,10 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -5768,7 +6670,10 @@
       <c r="D12" s="3">
         <v>1</v>
       </c>
-      <c r="E12" s="4"/>
+      <c r="E12" s="4">
+        <f>COUNTIF(B5:B46,1)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -5780,7 +6685,10 @@
       <c r="D13" s="3">
         <v>2</v>
       </c>
-      <c r="E13" s="4"/>
+      <c r="E13" s="4">
+        <f>COUNTIF(B5:B46,2)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -5792,7 +6700,10 @@
       <c r="D14" s="3">
         <v>3</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="4">
+        <f>COUNTIF(B5:B46,3)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -5804,7 +6715,10 @@
       <c r="D15" s="3">
         <v>4</v>
       </c>
-      <c r="E15" s="4"/>
+      <c r="E15" s="4">
+        <f>COUNTIF(B5:B46,4)</f>
+        <v>19</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -5816,7 +6730,10 @@
       <c r="D16" s="3">
         <v>5</v>
       </c>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4">
+        <f>COUNTIF(B5:B46,5)</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -6063,6 +6980,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Table de probalidad terminada
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\big_data\matematicas\analisis_estadistico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C943EF-923D-4C91-B8C5-63BCC539387A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FC471D-5408-4BC4-A535-2190AE8C177C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,8 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'4_Probabilidad'!$D$6:$D$8</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'4_Probabilidad'!$E$6:$E$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1525,6 +1527,267 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Probabilidad</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-ES" baseline="0"/>
+              <a:t> /Ventas por canal</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'4_Probabilidad'!$D$6:$D$8</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>App</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Web</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Tienda</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'4_Probabilidad'!$E$6:$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DF23-4A40-A904-0DF6460BAECB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1709,6 +1972,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -3204,6 +3507,525 @@
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -3381,6 +4203,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A536012-38AD-6E43-3603-6841D2FA2270}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Gráfico 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B537D5F-E705-8FD7-FFCB-9FB96F633BC6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6990,7 +7853,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" customWidth="1"/>
-    <col min="2" max="4" width="15.6640625" customWidth="1"/>
+    <col min="2" max="3" width="15.6640625" customWidth="1"/>
+    <col min="4" max="4" width="77.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7003,7 +7867,10 @@
       <c r="D3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="4">
+        <f>COUNTA(A5:A46)</f>
+        <v>42</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -7043,9 +7910,18 @@
       <c r="D6" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="7"/>
+      <c r="E6" s="4">
+        <f>COUNTIF(B5:B46,"App")</f>
+        <v>11</v>
+      </c>
+      <c r="F6" s="8">
+        <f>(E6/E3)</f>
+        <v>0.26190476190476192</v>
+      </c>
+      <c r="G6" s="7">
+        <f>F6</f>
+        <v>0.26190476190476192</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -7057,9 +7933,18 @@
       <c r="D7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="7"/>
+      <c r="E7" s="4">
+        <f>COUNTIF(B5:B46,"Web")</f>
+        <v>17</v>
+      </c>
+      <c r="F7" s="8">
+        <f>(E7/E3)</f>
+        <v>0.40476190476190477</v>
+      </c>
+      <c r="G7" s="7">
+        <f t="shared" ref="G7:G9" si="0">F7</f>
+        <v>0.40476190476190477</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -7071,9 +7956,18 @@
       <c r="D8" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="7"/>
+      <c r="E8" s="4">
+        <f>COUNTIF(B5:B46,"Tienda")</f>
+        <v>14</v>
+      </c>
+      <c r="F8" s="8">
+        <f>(E8/E3)</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G8" s="7">
+        <f t="shared" si="0"/>
+        <v>0.33333333333333331</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -7085,9 +7979,18 @@
       <c r="D9" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="7"/>
+      <c r="E9" s="4">
+        <f>SUM(E6:E8)</f>
+        <v>42</v>
+      </c>
+      <c r="F9" s="8">
+        <f>SUM(F6:F8)</f>
+        <v>1</v>
+      </c>
+      <c r="G9" s="7">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -7402,5 +8305,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>